<commit_message>
feat(phase-1): finalizacion oficial v1.3.0 de Fase 1 - Sistema PDV e Inventario WPC Bajio
</commit_message>
<xml_diff>
--- a/Validaciones/Checklist_Validacion_POS_Lambrin.xlsx
+++ b/Validaciones/Checklist_Validacion_POS_Lambrin.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyecto_PDV-CDC\Validaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39513A98-B4C9-4F6C-B222-8E0B46C66058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA9EF6F-DB9A-4DD2-83F6-B7A6B2E96B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="2595" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -2408,6 +2408,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2415,9 +2418,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2883,36 +2883,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
     </row>
     <row r="4" spans="1:8" ht="15">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="D4" s="14" t="s">
+      <c r="B4" s="15"/>
+      <c r="D4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="14"/>
+      <c r="E4" s="15"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B6" s="2">
         <f>'Fase 1'!B6</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>4</v>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="B9" s="2">
         <f>'Fase 1'!B9</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>7</v>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B11" s="2">
         <f>'Fase 1'!B11</f>
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>9</v>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B12" s="3">
         <f>'Fase 1'!B12</f>
-        <v>1.2987012987012988E-2</v>
+        <v>2.5974025974025976E-2</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -3043,76 +3043,76 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="15">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B6" s="2">
         <f>COUNTIF($I$15:$I$91,"Cumple")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="B9" s="2">
         <f>COUNTIF($I$15:$I$91,"En revisión")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="B11" s="2">
         <f>COUNTIF($I$15:$I$91,"Pendiente")</f>
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="B12" s="3">
         <f>IF(B5=0,0,(B6+B7*0.5)/B5)</f>
-        <v>1.2987012987012988E-2</v>
+        <v>2.5974025974025976E-2</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="33.950000000000003" customHeight="1">
@@ -3375,7 +3375,7 @@
         <v>41</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
@@ -3411,7 +3411,7 @@
         <v>54</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
@@ -3447,7 +3447,7 @@
         <v>41</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
@@ -8637,84 +8637,84 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="15">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>721</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="13" t="s">
         <v>722</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="13" t="s">
         <v>723</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="13" t="s">
         <v>724</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="13" t="s">
         <v>725</v>
       </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="13" t="s">
         <v>726</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="13" t="s">
         <v>727</v>
       </c>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="13" t="s">
         <v>728</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>